<commit_message>
Saving my local changes before pulling
</commit_message>
<xml_diff>
--- a/base/static/excel_sheet/category_excel_sheet.xlsx
+++ b/base/static/excel_sheet/category_excel_sheet.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Category_Name</t>
   </si>
@@ -50,15 +50,6 @@
   </si>
   <si>
     <t>Nutritious pet meals</t>
-  </si>
-  <si>
-    <t>ElectronicsElectronics</t>
-  </si>
-  <si>
-    <t>ewfbghn</t>
-  </si>
-  <si>
-    <t>sdfgrthnjym,kmng</t>
   </si>
 </sst>
 </file>
@@ -393,7 +384,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -448,22 +439,6 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>